<commit_message>
Internal накладная: fix Сумма to include margin, per corrected templates
The user caught a mistake in the two margin templates and resent corrected
copies: 'Сумма'/'Обшая сумма заказа' now spell out their own formula
(total_sum = sum_without_vat + vat_sum + margin_amount) rather than the
plain 'sum + vat' the customer-facing exports use — the internal накладная
is meant to show the marked-up total, not just base + VAT. Fixed
downloadOrderExcelWithMargin and downloadWeeklyInvoiceWithMarginExcel to
add margin into the line/order total; Прибыль (profit) itself is unchanged,
still just the margin amount.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/assets/templates/order-invoice-margin-template.xlsx
+++ b/src/assets/templates/order-invoice-margin-template.xlsx
@@ -72,9 +72,6 @@
     <t>Категория</t>
   </si>
   <si>
-    <t>[vat_amunt]</t>
-  </si>
-  <si>
     <t>Сумма без НДС</t>
   </si>
   <si>
@@ -106,6 +103,9 @@
   </si>
   <si>
     <t>Итого:[total_profit]</t>
+  </si>
+  <si>
+    <t>[total_sum=sum_without_vat+vat_sum+margin_amount]</t>
   </si>
 </sst>
 </file>
@@ -313,23 +313,11 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -340,15 +328,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -361,14 +340,35 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -709,10 +709,10 @@
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:24">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="24"/>
+      <c r="B2" s="20"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -721,10 +721,10 @@
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:24">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="26"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="2"/>
       <c r="D3" s="12"/>
       <c r="E3" s="7"/>
@@ -733,10 +733,10 @@
       <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:24" ht="15" customHeight="1">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="25"/>
+      <c r="B4" s="21"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -745,10 +745,10 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:24">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="25"/>
+      <c r="B5" s="21"/>
       <c r="C5" s="3"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -762,10 +762,10 @@
       <c r="O5" s="1"/>
     </row>
     <row r="6" spans="1:24">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="25"/>
+      <c r="B6" s="21"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -779,10 +779,10 @@
       <c r="O6" s="1"/>
     </row>
     <row r="7" spans="1:24" ht="15" customHeight="1">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="25"/>
+      <c r="B7" s="21"/>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
@@ -796,10 +796,10 @@
       <c r="O7" s="4"/>
     </row>
     <row r="8" spans="1:24" ht="15" customHeight="1" thickBot="1">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="25"/>
+      <c r="B8" s="21"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -821,26 +821,26 @@
         <v>2</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" s="30"/>
+      <c r="I9" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="H9" s="21"/>
-      <c r="I9" s="20" t="s">
+      <c r="J9" s="30"/>
+      <c r="K9" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="21"/>
-      <c r="K9" s="30" t="s">
-        <v>25</v>
-      </c>
-      <c r="L9" s="31"/>
+      <c r="L9" s="24"/>
     </row>
     <row r="10" spans="1:24" ht="34.5" thickBot="1">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="18" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="10" t="s">
@@ -852,24 +852,24 @@
       <c r="D10" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="34" t="s">
-        <v>19</v>
+      <c r="E10" s="19" t="s">
+        <v>18</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="32"/>
+      <c r="I10" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="J10" s="36"/>
+      <c r="K10" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="H10" s="28"/>
-      <c r="I10" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="23"/>
-      <c r="K10" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="L10" s="33"/>
+      <c r="L10" s="26"/>
       <c r="M10" s="9"/>
       <c r="N10" s="9"/>
       <c r="O10" s="9"/>
@@ -892,14 +892,14 @@
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
-      <c r="I11" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="J11" s="19"/>
-      <c r="K11" s="35" t="s">
-        <v>28</v>
-      </c>
-      <c r="L11" s="36"/>
+      <c r="I11" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="J11" s="34"/>
+      <c r="K11" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="L11" s="28"/>
       <c r="M11" s="9"/>
       <c r="N11" s="9"/>
       <c r="O11" s="9"/>

</xml_diff>